<commit_message>
Cap Pune-Bengaluru to 2 flights/airline; drop no-fare flights; per-section aviation dates
- max_per_airline (PNQ-BLR=2): keep flights spread across the day
- 'all' mode now drops flights with no bookable fare (removes Alliance Air on DEL-JAI)
- aviation panel resolves latest report date per section (MoCA updates cards
  at different times: traffic on 24th, load factor/on-time still 23rd)
- Captured 2026-07-25 (day 2): day-over-day deltas now populate

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aviation.xlsx
+++ b/aviation.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1431,6 +1431,486 @@
         </is>
       </c>
       <c r="H25" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Aircraft movements</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>5415</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>5,415</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Airport footfalls</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>808424</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>8,08,424</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Arriving Pax</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>403309</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>4,03,309</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Arriving flights</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2706</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2,706</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Departing Pax</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>405115</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>4,05,115</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Departing flights</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>2709</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2,709</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Aircraft movements</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1149</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1,149</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Airport footfalls</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>201655</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2,01,655</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Arriving Pax</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>104334</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>1,04,334</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Arriving flights</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>576</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Departing Pax</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>97321</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>97,321</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Departing flights</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>573</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>573</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
         <is>
           <t>civilaviation.gov.in</t>
         </is>
@@ -1532,7 +2012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1588,6 +2068,25 @@
         <v>560</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>24 July 2026</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>405115</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2709</v>
+      </c>
+      <c r="D3" t="n">
+        <v>97321</v>
+      </c>
+      <c r="E3" t="n">
+        <v>573</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Redesign: month-to-date averages, KPI row, aviation load-factor only, aesthetics
- Dashboard now shows month-to-date AVG price per flight/horizon with delta =
  last capture vs month avg (%). Same model for aviation.
- New KPI row: fare vs month avg, avg load factor (IndiGo/AI/Akasa), domestic &
  intl flights/day (month avg), flights/days captured, latest capture
- Aviation: month-avg per metric + delta; removed on-time %, load factor only w/ bars
- Validated palette (blue/orange series, proper ink/surface tokens), cleaner cards,
  tabular figures, light/dark; downloads moved to bottom
- Excel: keep full dump + add 'Dashboard' summary sheet (fares.xlsx & aviation.xlsx)
- Captured 2026-07-26 (day 3)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aviation.xlsx
+++ b/aviation.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Daily long" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Load factor" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Traffic" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daily long" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Load factor" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Traffic" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,7 +422,763 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>avg</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>last</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>pct_change</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Departing flights</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2660.67</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2652</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Departing Pax</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>397988</v>
+      </c>
+      <c r="E3" t="n">
+        <v>399206</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Arriving flights</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2660.67</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2661</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Arriving Pax</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>396825.33</v>
+      </c>
+      <c r="E5" t="n">
+        <v>400467</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Aircraft movements</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5321.33</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5313</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Airport footfalls</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>794813.33</v>
+      </c>
+      <c r="E7" t="n">
+        <v>799673</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Departing flights</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>568.33</v>
+      </c>
+      <c r="E8" t="n">
+        <v>572</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Departing Pax</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>96749.67</v>
+      </c>
+      <c r="E9" t="n">
+        <v>99230</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Arriving flights</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>571.33</v>
+      </c>
+      <c r="E10" t="n">
+        <v>577</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Arriving Pax</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>105218.67</v>
+      </c>
+      <c r="E11" t="n">
+        <v>108038</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Aircraft movements</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1139.67</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1149</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Airport footfalls</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>201968.33</v>
+      </c>
+      <c r="E13" t="n">
+        <v>207268</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>On Time Performance</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>On Time Performance</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Air India</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>88.84999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>88.84999999999999</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>On Time Performance</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SpiceJet</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>48</v>
+      </c>
+      <c r="E16" t="n">
+        <v>48</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>On Time Performance</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>72.22</v>
+      </c>
+      <c r="E17" t="n">
+        <v>72.22</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>On Time Performance</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Alliance Air</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>68</v>
+      </c>
+      <c r="E18" t="n">
+        <v>68</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>On Time Performance</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AKASA AIR</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="E19" t="n">
+        <v>92.31</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Passenger Load Factor</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>82.53</v>
+      </c>
+      <c r="E20" t="n">
+        <v>82.53</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Passenger Load Factor</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Air India</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="E21" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Passenger Load Factor</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SpiceJet</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Passenger Load Factor</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Air India Express</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>84.08</v>
+      </c>
+      <c r="E23" t="n">
+        <v>84.08</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Passenger Load Factor</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Alliance Air</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>50</v>
+      </c>
+      <c r="E24" t="n">
+        <v>50</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Passenger Load Factor</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>AKASA AIR</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>92.55</v>
+      </c>
+      <c r="E25" t="n">
+        <v>92.55</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1916,12 +2673,492 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Aircraft movements</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>5313</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>5,313</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Airport footfalls</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>799673</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>7,99,673</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Arriving Pax</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>400467</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>4,00,467</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Arriving flights</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>2661</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2,661</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Departing Pax</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>399206</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>3,99,206</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Domestic traffic</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Departing flights</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>2652</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2,652</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Aircraft movements</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1149</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>1,149</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Airport footfalls</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>207268</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2,07,268</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Arriving Pax</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>108038</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1,08,038</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Arriving flights</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>577</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>577</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Departing Pax</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>99230</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>99,230</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>International traffic</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Departing flights</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>572</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>572</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>civilaviation.gov.in</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2006,13 +3243,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2087,6 +3324,25 @@
         <v>573</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>25 July 2026</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>399206</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2652</v>
+      </c>
+      <c r="D4" t="n">
+        <v>99230</v>
+      </c>
+      <c r="E4" t="n">
+        <v>572</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>